<commit_message>
minor changes in v5 and v6 and failed batch requests
</commit_message>
<xml_diff>
--- a/output_files/Results_AoA_f_t_2000.xlsx
+++ b/output_files/Results_AoA_f_t_2000.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,7 +454,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>radioescucha</t>
+          <t>esprit</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,18 +463,18 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10.5</v>
+        <v>5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Dictionary_on_web</t>
+          <t>fundeu_dic</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>párrocos</t>
+          <t>sanedrín</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -483,18 +483,18 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Marul et al. (2014)</t>
+          <t>Dictionary_on_web</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>encurrujarse</t>
+          <t>acelajado</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>8.5</v>
+        <v>12.5</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>universidad pontificia</t>
+          <t>honorable</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,18 +523,18 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>18.5</v>
+        <v>10.5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Marul et al. (2014)</t>
+          <t>Dictionary_on_web</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>temporalista</t>
+          <t>ñandubay</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -543,18 +543,18 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>10.5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>fundeu_dic</t>
+          <t>Dictionary_on_web</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>primadona</t>
+          <t>galindo</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -563,18 +563,18 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>fundeu_dic</t>
+          <t>Dictionary_on_web</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>localización</t>
+          <t>memoriona</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -587,14 +587,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Dictionary_on_web</t>
+          <t>fundeu_dic</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>citocentro</t>
+          <t>esmola</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -603,18 +603,18 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>12.5</v>
+        <v>6.5</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>fundeu_dic</t>
+          <t>Dictionary_on_web</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>sudorípara</t>
+          <t>zuma</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -623,7 +623,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>10.5</v>
+        <v>5</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>encomendero</t>
+          <t>vellorita</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -643,9 +643,407 @@
         </is>
       </c>
       <c r="C11" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>almodón</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>RAE_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>tabarés</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>fundeu_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>presea</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>comedición</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>RAE_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>aducir</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>arqueoturismo</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
         <v>15</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>fundeu_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>pastrija</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>RAE_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>quillango</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>culo</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>reagrupar</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>iusnaturalismo</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>10.98</v>
+      </c>
+      <c r="C22" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>fundeu_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sacrificarse</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Abella (2020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>torio</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>tandero</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>RAE_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>oncológico</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>quater</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>fundeu_dic</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>anegar</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>copudo</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>toletazo</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Dictionary_on_web</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>contraria</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D31" t="inlineStr">
         <is>
           <t>Dictionary_on_web</t>
         </is>
@@ -662,7 +1060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -722,6 +1120,101 @@
         <v>9</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>